<commit_message>
feat(sg): allow certain cantonal service to invite each other
Related to https://jira.sg.ch/browse/EBAU-296
</commit_message>
<xml_diff>
--- a/django/kt_sg/import/Services_SG.xlsx
+++ b/django/kt_sg/import/Services_SG.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="169">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -292,24 +292,42 @@
     <t xml:space="preserve">AFU-BS-AR Abfall und Rohstoffe</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-bs-ar</t>
+  </si>
+  <si>
     <t xml:space="preserve">{"distribution-group": "bud"}</t>
   </si>
   <si>
     <t xml:space="preserve">AFU-BS-BA Boden und Altlasten</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-bs-ba</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-BS-LW Landwirtschaftlicher Umweltschutz</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-bs-lw</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-IG-B1 Betriebe 1</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-ig-b1</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-IG-B2 Betriebe 2</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-ig-b2</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-IG-LU Luftqualität</t>
   </si>
   <si>
+    <t xml:space="preserve">afu-ig-lu</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-RU-RD Rechtsdienst</t>
   </si>
   <si>
@@ -367,7 +385,13 @@
     <t xml:space="preserve">AWE-GG-AW Abwasser</t>
   </si>
   <si>
+    <t xml:space="preserve">awe-gg-aw</t>
+  </si>
+  <si>
     <t xml:space="preserve">AWE-GG-GW Grundwasser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">awe-gg-gw</t>
   </si>
   <si>
     <t xml:space="preserve">AWE-GG-WK Wasserkraft</t>
@@ -790,7 +814,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.77"/>
@@ -1918,11 +1942,14 @@
       <c r="B78" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="C78" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="J78" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,13 +1957,16 @@
         <v>3</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="J79" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L79" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1944,13 +1974,16 @@
         <v>3</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="J80" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L80" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1958,13 +1991,16 @@
         <v>3</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="J81" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L81" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1972,13 +2008,16 @@
         <v>3</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>94</v>
+        <v>98</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="J82" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1986,13 +2025,16 @@
         <v>3</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="J83" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L83" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2000,13 +2042,13 @@
         <v>3</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J84" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L84" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2014,13 +2056,13 @@
         <v>3</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J85" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2028,13 +2070,13 @@
         <v>3</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="J86" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L86" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2042,13 +2084,13 @@
         <v>3</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="J87" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L87" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,13 +2098,13 @@
         <v>3</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J88" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L88" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2070,13 +2112,13 @@
         <v>3</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="J89" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L89" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2084,13 +2126,13 @@
         <v>3</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="J90" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L90" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2098,13 +2140,13 @@
         <v>3</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="J91" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L91" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2112,13 +2154,13 @@
         <v>3</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="J92" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L92" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2126,13 +2168,13 @@
         <v>3</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="J93" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L93" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2140,13 +2182,13 @@
         <v>3</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="J94" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L94" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2154,13 +2196,13 @@
         <v>3</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="J95" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2168,13 +2210,13 @@
         <v>3</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="J96" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2182,13 +2224,13 @@
         <v>3</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="J97" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,13 +2238,13 @@
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J98" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L98" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2210,13 +2252,13 @@
         <v>3</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J99" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L99" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2224,13 +2266,13 @@
         <v>3</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="J100" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L100" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2238,13 +2280,13 @@
         <v>3</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="J101" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L101" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2252,13 +2294,16 @@
         <v>3</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="J102" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L102" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2266,13 +2311,16 @@
         <v>3</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>115</v>
+        <v>122</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="J103" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L103" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2280,13 +2328,13 @@
         <v>3</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J104" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L104" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2294,13 +2342,13 @@
         <v>3</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="J105" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L105" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2308,13 +2356,13 @@
         <v>3</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="J106" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L106" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2322,13 +2370,13 @@
         <v>3</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J107" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L107" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2336,13 +2384,13 @@
         <v>3</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="J108" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L108" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2350,13 +2398,13 @@
         <v>3</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J109" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L109" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2364,13 +2412,13 @@
         <v>3</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="J110" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L110" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2378,13 +2426,13 @@
         <v>3</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="J111" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L111" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2392,13 +2440,13 @@
         <v>3</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="J112" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L112" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2406,13 +2454,13 @@
         <v>3</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="J113" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L113" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2420,13 +2468,13 @@
         <v>3</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J114" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L114" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2434,13 +2482,13 @@
         <v>3</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="J115" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L115" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,13 +2496,13 @@
         <v>3</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="J116" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L116" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2462,13 +2510,13 @@
         <v>3</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="J117" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L117" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2476,13 +2524,13 @@
         <v>3</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="J118" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L118" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2490,13 +2538,13 @@
         <v>3</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="J119" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L119" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2504,13 +2552,13 @@
         <v>3</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="J120" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L120" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2518,13 +2566,13 @@
         <v>3</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="J121" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L121" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2532,13 +2580,13 @@
         <v>3</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="J122" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L122" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2546,13 +2594,13 @@
         <v>3</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="J123" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L123" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2560,13 +2608,13 @@
         <v>3</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="J124" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L124" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2574,13 +2622,13 @@
         <v>3</v>
       </c>
       <c r="B125" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J125" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="J125" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L125" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,13 +2636,13 @@
         <v>3</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="J126" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L126" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2602,13 +2650,13 @@
         <v>3</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="J127" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L127" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2616,13 +2664,13 @@
         <v>3</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="J128" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L128" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2630,13 +2678,13 @@
         <v>3</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="J129" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L129" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2644,13 +2692,13 @@
         <v>3</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J130" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L130" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2658,7 +2706,7 @@
         <v>4</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="J131" s="1" t="n">
         <v>0</v>
@@ -2669,7 +2717,7 @@
         <v>4</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="J132" s="1" t="n">
         <v>0</v>
@@ -2680,7 +2728,7 @@
         <v>5</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J133" s="1" t="n">
         <v>0</v>
@@ -2691,7 +2739,7 @@
         <v>5</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="J134" s="1" t="n">
         <v>0</v>
@@ -2702,7 +2750,7 @@
         <v>5</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="J135" s="1" t="n">
         <v>0</v>
@@ -2713,7 +2761,7 @@
         <v>5</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="J136" s="1" t="n">
         <v>0</v>
@@ -2724,7 +2772,7 @@
         <v>5</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="J137" s="1" t="n">
         <v>0</v>
@@ -2735,7 +2783,7 @@
         <v>5</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="J138" s="1" t="n">
         <v>0</v>
@@ -2746,7 +2794,7 @@
         <v>5</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="J139" s="1" t="n">
         <v>0</v>
@@ -2757,7 +2805,7 @@
         <v>5</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="J140" s="1" t="n">
         <v>0</v>
@@ -2768,7 +2816,7 @@
         <v>5</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="J141" s="1" t="n">
         <v>0</v>
@@ -2779,7 +2827,7 @@
         <v>5</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="J142" s="1" t="n">
         <v>0</v>
@@ -2790,7 +2838,7 @@
         <v>5</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="J143" s="1" t="n">
         <v>0</v>
@@ -2801,7 +2849,7 @@
         <v>5</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="J144" s="1" t="n">
         <v>0</v>
@@ -2812,34 +2860,12 @@
         <v>5</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J145" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>